<commit_message>
Update Task 5 Equality Table.xlsx
</commit_message>
<xml_diff>
--- a/Task 5 Equality Table.xlsx
+++ b/Task 5 Equality Table.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e5f33f035f15c272/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tirth\Documents\GitHub\demo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="11_59442BC3ADFCDE8967613BC65B0958EC902A0173" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA808541-4679-4B4F-A6EA-21A26A0340E6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4095B282-C1CC-4EB6-84A5-E83882306044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -159,10 +159,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>